<commit_message>
feat: Add comprehensive family management, including API integration, Excel import/export, and a new projects section for campaigns.
</commit_message>
<xml_diff>
--- a/families_test_upload.xlsx
+++ b/families_test_upload.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet name="families" sheetId="1" r:id="rId1"/>
     <sheet name="members" sheetId="2" r:id="rId2"/>
+    <sheet name="README" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -398,19 +399,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K3"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" customWidth="1"/>
-    <col min="9" max="9" width="22.83203125" customWidth="1"/>
-    <col min="10" max="10" width="22.83203125" customWidth="1"/>
-    <col min="11" max="11" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="11" max="11" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -450,7 +451,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>آل السيد</v>
+        <v>Al-Sayed Family</v>
       </c>
       <c r="B2" t="str">
         <v>123456789</v>
@@ -474,10 +475,10 @@
         <v>T-12</v>
       </c>
       <c r="I2" t="str">
-        <v>القطاع أ</v>
+        <v>Sector A, Camp 1</v>
       </c>
       <c r="J2" t="str">
-        <v>لا ملاحظات</v>
+        <v>No special notes</v>
       </c>
       <c r="K2" t="str">
         <v>male</v>
@@ -485,7 +486,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>محمد</v>
+        <v>Mohamed Family</v>
       </c>
       <c r="B3" t="str">
         <v>223344556</v>
@@ -496,9 +497,6 @@
       <c r="D3" t="str">
         <v>+201112223334</v>
       </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
       <c r="F3">
         <v>2</v>
       </c>
@@ -509,7 +507,7 @@
         <v>T-15</v>
       </c>
       <c r="I3" t="str">
-        <v>القطاع ب</v>
+        <v>Sector B, Camp 1</v>
       </c>
       <c r="J3" t="str">
         <v/>
@@ -518,60 +516,25 @@
         <v>male</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>الأحمدي</v>
-      </c>
-      <c r="B4" t="str">
-        <v>334455667</v>
-      </c>
-      <c r="C4" t="str">
-        <v>1990-03-08</v>
-      </c>
-      <c r="D4" t="str">
-        <v>+966500000001</v>
-      </c>
-      <c r="E4" t="str">
-        <v>+966500000002</v>
-      </c>
-      <c r="F4">
-        <v>4</v>
-      </c>
-      <c r="G4">
-        <v>2</v>
-      </c>
-      <c r="H4" t="str">
-        <v>T-20</v>
-      </c>
-      <c r="I4" t="str">
-        <v>القطاع ج</v>
-      </c>
-      <c r="J4" t="str">
-        <v>عائلة ضعيفة</v>
-      </c>
-      <c r="K4" t="str">
-        <v>male</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H3"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="26.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+    <col min="4" max="4" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="26.83203125" customWidth="1"/>
+    <col min="6" max="6" width="26.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -605,22 +568,22 @@
         <v>123456789</v>
       </c>
       <c r="B2" t="str">
-        <v>أحمد السيد</v>
+        <v>Sara Al-Sayed</v>
       </c>
       <c r="C2" t="str">
-        <v>male</v>
+        <v>female</v>
       </c>
       <c r="D2" t="str">
-        <v>2005-08-10</v>
+        <v>2010-02-15</v>
       </c>
       <c r="E2" t="str">
-        <v>987654321</v>
+        <v>876543219</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>Asthma</v>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -628,137 +591,172 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>123456789</v>
+        <v>223344556</v>
       </c>
       <c r="B3" t="str">
-        <v>سارة السيد</v>
+        <v>Fatma Ali</v>
       </c>
       <c r="C3" t="str">
         <v>female</v>
       </c>
       <c r="D3" t="str">
-        <v>2010-02-15</v>
+        <v>2003-07-19</v>
       </c>
       <c r="E3" t="str">
-        <v>876543219</v>
+        <v>445566778</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3" t="str">
-        <v>ربو</v>
+        <v>Diabetes</v>
       </c>
       <c r="H3" t="str">
         <v/>
       </c>
     </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A25"/>
+  <cols>
+    <col min="1" max="1" width="70.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>📋 HOW TO USE THIS TEMPLATE</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>SHEET 1 — families</v>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>223344556</v>
-      </c>
-      <c r="B4" t="str">
-        <v>محمد علي</v>
-      </c>
-      <c r="C4" t="str">
-        <v>male</v>
-      </c>
-      <c r="D4" t="str">
-        <v>2000-03-22</v>
-      </c>
-      <c r="E4" t="str">
-        <v>334455001</v>
-      </c>
-      <c r="F4">
-        <v>3</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v/>
+        <v xml:space="preserve">  • One row per FAMILY HEAD.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>334455667</v>
-      </c>
-      <c r="B5" t="str">
-        <v>فاطمة الأحمدي</v>
-      </c>
-      <c r="C5" t="str">
-        <v>female</v>
-      </c>
-      <c r="D5" t="str">
-        <v>1992-07-01</v>
-      </c>
-      <c r="E5" t="str">
-        <v>334455668</v>
-      </c>
-      <c r="F5">
-        <v>2</v>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
-        <v/>
+        <v xml:space="preserve">  • The head is automatically added as the first member (relationship_id=1).</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>334455667</v>
-      </c>
-      <c r="B6" t="str">
-        <v>عمر الأحمدي</v>
-      </c>
-      <c r="C6" t="str">
-        <v>male</v>
-      </c>
-      <c r="D6" t="str">
-        <v>2012-01-15</v>
-      </c>
-      <c r="E6" t="str">
-        <v>334455669</v>
-      </c>
-      <c r="F6">
-        <v>3</v>
-      </c>
-      <c r="G6" t="str">
-        <v>سكري</v>
-      </c>
-      <c r="H6" t="str">
-        <v/>
+        <v xml:space="preserve">  • You do NOT need to add the head in the members sheet.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>334455667</v>
-      </c>
-      <c r="B7" t="str">
-        <v>نور الأحمدي</v>
-      </c>
-      <c r="C7" t="str">
-        <v>female</v>
-      </c>
-      <c r="D7" t="str">
-        <v>2015-09-20</v>
-      </c>
-      <c r="E7" t="str">
-        <v>334455670</v>
-      </c>
-      <c r="F7">
-        <v>3</v>
-      </c>
-      <c r="G7" t="str">
         <v/>
       </c>
-      <c r="H7" t="str">
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>SHEET 2 — members</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v xml:space="preserve">  • One row per ADDITIONAL MEMBER (not the head).</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v xml:space="preserve">  • Link each member to their family using family_national_id.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v xml:space="preserve">  • Multiple rows with the same family_national_id = multiple extra members.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v xml:space="preserve">  • Example: family with 3 total members → 1 row in families + 2 rows in members.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
         <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>relationship_id values:</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v xml:space="preserve">  1 = رب الأسرة (head) — auto-added, DO NOT add here</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v xml:space="preserve">  2 = زوجة / زوج</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v xml:space="preserve">  3 = ابن / ابنة</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v xml:space="preserve">  4 = أخ / أخت</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v xml:space="preserve">  5 = آخر</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>marital_status_id values:</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v xml:space="preserve">  1 = أعزب</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v xml:space="preserve">  2 = متزوج</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v xml:space="preserve">  3 = مطلق</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v xml:space="preserve">  4 = أرمل</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>